<commit_message>
feat(F-NAR-019): ATOM-EMO.LEX.001-03 Nina et la cerise du matin
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-EMO.LEX.001-03.xlsx
+++ b/stories/arbres/ATOM-EMO.LEX.001-03.xlsx
@@ -671,7 +671,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>jardin, cerisier</t>
+          <t>jardin, cerisier, portail, cerise, noyau, tuteur, herbe, bois, soleil, panier</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Nina pousse le portail. Elle cueille une cerise. Elle dit sa joie. Elle la partage avec papa et maman.</t>
+          <t>L'air près du cerisier sent le sucre. Sur le bois, un éclat de tuteur luit. Nina veut la cerise, maintenant. Branche trop haute, doigts qui glissent. Sourire parti, poitrine, papa accroupi. Une cerise plus bas. Un sourire arrive. Je suis contente. Partage, merci vécu. Deuxième ruse : jus qui coule, branche trop haute, oiseau. Elle refuse de foncer. Noyau, portail. Un éclat de tuteur tient sur le bois.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Le portail de bois claque tout doux. Une abeille passe près des feuilles. L'herbe est mouillée de rosée. Ça sent le vert et le sucre. Un oiseau picore près du bac. Le bois du portail sent la rosée. La maison est derrière, encore un peu endormie. Papa porte un petit panier d'osier. Maman ferme le portail derrière eux. Tu as vu le cerisier, Nina ? Il est tout rouge ! Les cerises sont mûres ce matin. En ce moment, Nina marche dans l'herbe. Ses bottes font un bruit mou. Le matin est clair, tout clair. Le cerisier fait une ombre ronde. Une cerise brille, toute seule, à hauteur de main. Nina la touche du bout du doigt. La peau est lisse et un peu froide. Tu peux la cueillir tout doucement. Nina la détache. La queue reste entre ses doigts. La cerise sent le sucre. Parce que la cerise est là, ses joues deviennent chaudes. Son ventre est léger, comme une bulle. Un sourire arrive. Je suis contente. C'est de la joie. Tu as nommé ta joie. Bravo, Nina. On peut partager ? Oui. On partage. Nina tend la cerise vers papa. Merci. Un tout petit bout pour moi. Papa croque un tout petit bout. Nina croque un tout petit bout. Le jus est rouge et doux. Maman, un bout pour toi. Merci, ma grande. Tu m'invites. C'est gentil. Ils restent sous le cerisier. Une feuille tombe, toute légère. Tu as encore de la joie ? Oui, papa. Je suis contente. Le panier attend, vide et prêt.</t>
+          <t>L'air près du cerisier sent le sucre. Ça sent le sucre, papa. Tu le sens, le sucre, Nina ? Oui, papa. Le portail de bois reste un peu ouvert. Il est ouvert, maman. Tu entends le bois, Nina ? Il claque, maman. L'herbe froide mouille les pieds de Nina. Elle est mouillée. Elle pique un peu, Nina ? Un peu, maman. Le tuteur tient une branche basse, près du portail. Il est en bois. Tu le vois, le tuteur ? Oui, papa. Sur le bois, un éclat de tuteur luit. Il brille, maman. Tu le vois, le petit point ? Oui, un petit point. Papa pose le panier près de l'herbe. Le panier est là. Il attend, près de nous. Oui. Une cerise rouge attend trop haut. Elle est rouge ! Tu la veux, Nina ? Oui, papa. Le soleil chauffe la peau lisse. Elle brille. La cerise est loin, Nina ? Un peu loin. En ce moment, Nina lève les deux mains. Je veux la cerise, maintenant ! Tout de suite ? Oui, papa. Nina saute trop vite vers la branche. Ses doigts glissent sur la peau lisse. La cerise reste trop haute. Oh. Le sourire de Nina disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent sans place. Sa poitrine va trop vite. Elle est trop haute, Nina ? Oui, papa. Tes joues sont chaudes, Nina ? Un peu, maman. L'éclat de tuteur tremble, puis tient. Papa s'accroupit à la même hauteur, sans parler. Tu vois une autre, Nina ? Là, plus bas. Une cerise plus basse brille à hauteur de main. Nina la touche du bout du doigt. Elle est froide. Tu la cueilles, Nina ? Oui. Nina détache la cerise plus basse, sans se presser. La queue reste entre ses doigts. Elle est lourde. Elle tient dans ta main ? Oui, papa. La cerise sent le sucre. Ses joues deviennent chaudes. Son ventre est léger, comme une bulle. Ça chatouille. Tes épaules se relèvent, Nina ? Un peu, maman. Un sourire arrive.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Le portail de bois claque tout doux. Une abeille passe près des feuilles. L'herbe est mouillée de rosée. Ça sent le vert et le sucre. Un oiseau picore près du bac. Le bois du portail sent la rosée. La maison est derrière, encore un peu endormie. Papa porte un petit panier d'osier. Maman ferme le portail derrière eux. Tu as vu le cerisier, Nina ? Il est tout rouge ! Les cerises sont mûres ce matin. En ce moment, Nina marche dans l'herbe. Ses bottes font un bruit mou. Le matin est clair, tout clair. Le cerisier fait une ombre ronde. Une cerise brille, toute seule, à hauteur de main. Nina la touche du bout du doigt. La peau est lisse et un peu froide. Tu peux la cueillir tout doucement. Nina la détache. La queue reste entre ses doigts. La cerise sent le sucre. Parce que la cerise est là, ses joues deviennent chaudes. Son ventre est léger, comme une bulle. Un sourire arrive. Je suis contente. C'est de la joie. Tu as nommé ta joie. Bravo, Nina. On peut partager ? Oui. On partage. Nina tend la cerise vers papa. Merci. Un tout petit bout pour moi. Papa croque un tout petit bout. Nina croque un tout petit bout. Le jus est rouge et doux. Maman, un bout pour toi. Merci, ma grande. Tu m'invites. C'est gentil. Ils restent sous le cerisier. Une feuille tombe, toute légère. Tu as encore de la joie ? Oui, papa. Je suis contente. Le panier attend, vide et prêt.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;L'air près du cerisier sent le sucre. Ça sent le sucre, papa. Tu le sens, le sucre, Nina ? Oui, papa. Le portail de bois reste un peu ouvert. Il est ouvert, maman. Tu entends le bois, Nina ? Il claque, maman. L'herbe froide mouille les pieds de Nina. Elle est mouillée. Elle pique un peu, Nina ? Un peu, maman. Le tuteur tient une branche basse, près du portail. Il est en bois. Tu le vois, le tuteur ? Oui, papa. Sur le bois, un &lt;emphasis level="moderate"&gt;éclat de tuteur&lt;/emphasis&gt; luit. Il brille, maman. Tu le vois, le petit point ? Oui, un petit point. Papa pose le panier près de l'herbe. Le panier est là. Il attend, près de nous. Oui. Une cerise rouge attend trop haut. Elle est rouge ! Tu la veux, Nina ? Oui, papa. Le soleil chauffe la peau lisse. Elle brille. La cerise est loin, Nina ? Un peu loin. En ce moment, Nina lève les deux mains. Je veux la cerise, maintenant ! Tout de suite ? Oui, papa. Nina saute trop vite vers la branche. Ses doigts glissent sur la peau lisse. La cerise reste trop haute. Oh. Le sourire de Nina disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent sans place. Sa poitrine va trop vite. Elle est trop haute, Nina ? Oui, papa. Tes joues sont chaudes, Nina ? Un peu, maman. L'éclat de tuteur tremble, puis tient. Papa s'accroupit à la même hauteur, sans parler. Tu vois une autre, Nina ? Là, plus bas. Une cerise plus basse brille à hauteur de main. Nina la touche du bout du doigt. Elle est froide. Tu la cueilles, Nina ? Oui. Nina détache la cerise plus basse, sans se presser. La queue reste entre ses doigts. Elle est lourde. Elle tient dans ta main ? Oui, papa. La cerise sent le sucre. Ses joues deviennent chaudes. Son ventre est léger, comme une bulle. Ça chatouille. Tes épaules se relèvent, Nina ? Un peu, maman. Un sourire arrive.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Emma marche dans le jardin. Papa est là, près du cerisier. Le soleil est doux. Emma voit une cerise rouge. Elle la cueille tout doucement. La cerise sent le sucre. Parce que la cerise est là, Emma sent ses joues chaudes. Son ventre est léger. Un sourire arrive. Emma dit : je suis &lt;emphasis&gt;content&lt;/emphasis&gt;e. Papa dit : c'est de la joie. Être content, c'est bien. Parce qu'elle a de la joie, Emma veut partager. Elle tend la cerise. Elle dit : on peut partager. Papa prend un tout petit bout. Emma prend un tout petit bout. Ils sourient ensemble. Emma dit encore : je suis contente. La joie est là, dans le jardin. Papa lui prend la main. [pause]</t>
+          <t>L'air près du cerisier sent le sucre. Ça sent le sucre, papa. Tu le sens, le sucre, Nina ? Oui, papa. Le portail de bois reste un peu ouvert. Il est ouvert, maman. Tu entends le bois, Nina ? Il claque, maman. L'herbe froide mouille les pieds de Nina. Elle est mouillée. Elle pique un peu, Nina ? Un peu, maman. Le tuteur tient une branche basse, près du portail. Il est en bois. Tu le vois, le tuteur ? Oui, papa. Sur le bois, un &lt;emphasis&gt;éclat de tuteur&lt;/emphasis&gt; luit. Il brille, maman. Tu le vois, le petit point ? Oui, un petit point. Papa pose le panier près de l'herbe. Le panier est là. Il attend, près de nous. Oui. Une cerise rouge attend trop haut. Elle est rouge ! Tu la veux, Nina ? Oui, papa. Le soleil chauffe la peau lisse. Elle brille. La cerise est loin, Nina ? Un peu loin. En ce moment, Nina lève les deux mains. Je veux la cerise, maintenant ! Tout de suite ? Oui, papa. Nina saute trop vite vers la branche. Ses doigts glissent sur la peau lisse. La cerise reste trop haute. Oh. Le sourire de Nina disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent sans place. Sa poitrine va trop vite. Elle est trop haute, Nina ? Oui, papa. Tes joues sont chaudes, Nina ? Un peu, maman. L'éclat de tuteur tremble, puis tient. Papa s'accroupit à la même hauteur, sans parler. Tu vois une autre, Nina ? Là, plus bas. Une cerise plus basse brille à hauteur de main. Nina la touche du bout du doigt. Elle est froide. Tu la cueilles, Nina ? Oui. Nina détache la cerise plus basse, sans se presser. La queue reste entre ses doigts. Elle est lourde. Elle tient dans ta main ? Oui, papa. La cerise sent le sucre. Ses joues deviennent chaudes. Son ventre est léger, comme une bulle. Ça chatouille. Tes épaules se relèvent, Nina ? Un peu, maman. Un sourire arrive. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,10 +1249,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.18</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>content</t>
+          <t>éclat de tuteur</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1321,58 +1321,86 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis joie_naissante; intensite=2; destinataire=enfant; sous_texte=elle_veut_la_cerise_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun puis léger; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Le portail de bois claque tout doux.
-narrateur|Une abeille passe près des feuilles.
-narrateur|L'herbe est mouillée de rosée.
-narrateur|Ça sent le vert et le sucre.
-narrateur|Un oiseau picore près du bac.
-narrateur|Le bois du portail sent la rosée.
-narrateur|La maison est derrière, encore un peu endormie.
-narrateur|Papa porte un petit panier d'osier.
-narrateur|Maman ferme le portail derrière eux.
-papa|Tu as vu le cerisier, Nina ?
-enfant-f|Il est tout rouge !
-maman|Les cerises sont mûres ce matin.
-narrateur|En ce moment, Nina marche dans l'herbe.
-narrateur|Ses bottes font un bruit mou.
-narrateur|Le matin est clair, tout clair.
-narrateur|Le cerisier fait une ombre ronde.
-narrateur|Une cerise brille, toute seule, à hauteur de main.
+          <t>narrateur|L'air près du cerisier sent le sucre.
+enfant-f|Ça sent le sucre, papa.
+papa|Tu le sens, le sucre, Nina ?
+enfant-f|Oui, papa.
+narrateur|Le portail de bois reste un peu ouvert.
+enfant-f|Il est ouvert, maman.
+maman|Tu entends le bois, Nina ?
+enfant-f|Il claque, maman.
+narrateur|L'herbe froide mouille les pieds de Nina.
+enfant-f|Elle est mouillée.
+maman|Elle pique un peu, Nina ?
+enfant-f|Un peu, maman.
+narrateur|Le tuteur tient une branche basse, près du portail.
+enfant-f|Il est en bois.
+papa|Tu le vois, le tuteur ?
+enfant-f|Oui, papa.
+narrateur|Sur le bois, un éclat de tuteur luit.
+enfant-f|Il brille, maman.
+maman|Tu le vois, le petit point ?
+enfant-f|Oui, un petit point.
+narrateur|Papa pose le panier près de l'herbe.
+enfant-f|Le panier est là.
+papa|Il attend, près de nous.
+enfant-f|Oui.
+narrateur|Une cerise rouge attend trop haut.
+enfant-f|Elle est rouge !
+papa|Tu la veux, Nina ?
+enfant-f|Oui, papa.
+narrateur|Le soleil chauffe la peau lisse.
+enfant-f|Elle brille.
+maman|La cerise est loin, Nina ?
+enfant-f|Un peu loin.
+narrateur|En ce moment, Nina lève les deux mains.
+enfant-f|Je veux la cerise, maintenant !
+papa|Tout de suite ?
+enfant-f|Oui, papa.
+narrateur|Nina saute trop vite vers la branche.
+narrateur|Ses doigts glissent sur la peau lisse.
+narrateur|La cerise reste trop haute.
+enfant-f|Oh.
+narrateur|Le sourire de Nina disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent sans place.
+narrateur|Sa poitrine va trop vite.
+papa|Elle est trop haute, Nina ?
+enfant-f|Oui, papa.
+maman|Tes joues sont chaudes, Nina ?
+enfant-f|Un peu, maman.
+narrateur|L'éclat de tuteur tremble, puis tient.
+narrateur|Papa s'accroupit à la même hauteur, sans parler.
+papa|Tu vois une autre, Nina ?
+enfant-f|Là, plus bas.
+narrateur|Une cerise plus basse brille à hauteur de main.
 narrateur|Nina la touche du bout du doigt.
-narrateur|La peau est lisse et un peu froide.
-papa|Tu peux la cueillir tout doucement.
-narrateur|Nina la détache. La queue reste entre ses doigts.
+enfant-f|Elle est froide.
+maman|Tu la cueilles, Nina ?
+enfant-f|Oui.
+narrateur|Nina détache la cerise plus basse, sans se presser.
+narrateur|La queue reste entre ses doigts.
+enfant-f|Elle est lourde.
+papa|Elle tient dans ta main ?
+enfant-f|Oui, papa.
 narrateur|La cerise sent le sucre.
-narrateur|Parce que la cerise est là, ses joues deviennent chaudes.
+narrateur|Ses joues deviennent chaudes.
 narrateur|Son ventre est léger, comme une bulle.
-narrateur|Un sourire arrive.
-enfant-f|Je suis contente.
-papa|C'est de la joie.
-papa|Tu as nommé ta joie.
-maman|Bravo, Nina.
-enfant-f|On peut partager ?
-maman|Oui. On partage.
-narrateur|Nina tend la cerise vers papa.
-papa|Merci. Un tout petit bout pour moi.
-narrateur|Papa croque un tout petit bout.
-narrateur|Nina croque un tout petit bout.
-narrateur|Le jus est rouge et doux.
-enfant-f|Maman, un bout pour toi.
-maman|Merci, ma grande.
-maman|Tu m'invites. C'est gentil.
-narrateur|Ils restent sous le cerisier.
-narrateur|Une feuille tombe, toute légère.
-papa|Tu as encore de la joie ?
-enfant-f|Oui, papa. Je suis contente.
-narrateur|Le panier attend, vide et prêt.</t>
+enfant-f|Ça chatouille.
+maman|Tes épaules se relèvent, Nina ?
+enfant-f|Un peu, maman.
+narrateur|Un sourire arrive.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>oiseau</t>
+          <t>jardin,cerisier</t>
         </is>
       </c>
     </row>
@@ -1404,12 +1432,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Nina sourit. Que dit-elle ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;&lt;emphasis level="moderate"&gt;Nina&lt;/emphasis&gt; sourit. Que dit-elle ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Emma sourit. Que dit-elle ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;&lt;emphasis&gt;Nina&lt;/emphasis&gt; sourit. Que dit-elle ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1434,7 +1462,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Emma sent de la joie. Que dit-elle ?</t>
+          <t>Nina sent de la joie. Que dit-elle ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1472,7 +1500,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1483,7 +1511,7 @@
         <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.3</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1498,34 +1526,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>Nina</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1540,22 +1572,23 @@
         <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=nina_sourit_que_dit_elle; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Nina sourit. Que dit-elle ?</t>
+          <t>narrateur|Nina sourit.
+narrateur|Que dit-elle ?</t>
         </is>
       </c>
     </row>
@@ -1582,17 +1615,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Nina a encore un peu de jus au doigt. C'est de la joie. Oui. Tu es contente. Et tu as partagé ta cerise. Tu as fini ton petit bout ? Oui. Nina essuie ses doigts sur l'herbe. Le cerisier fait encore de l'ombre.</t>
+          <t>Nina tient la cerise contre sa paume, tout près. Je suis contente. Tu le dis, Nina ? Oui, papa. Ses joues restent chaudes. Le ventre de Nina se desserre. On partage ? Tu veux tendre la cerise ? Oui, maman. Nina avance la cerise trop vite. Elle ouvre la bouche, trop large. Puis elle s'arrête. Nina refuse de foncer. Personne ne parle. Elle observe la cerise, un instant. Elle écoute le jardin. Nina tend la cerise vers papa. Papa prend un tout petit bout. Merci, Nina. Papa a vu le geste, sous l'arbre. Le jus est rouge. Il colle aux doigts, Nina ? Un peu, maman. Nina croque un tout petit bout. C'est sucré. Tu le sens, le sucre ? Oui, papa. Tes lèvres sont rouges, Nina ? Un peu, maman. Le ventre de Nina reste léger. Maman, un bout pour toi. Tu m'invites, Nina ? Oui. Maman attend, la main ouverte. La cerise est petite, Nina ? Oui, papa. Ils restent sous le cerisier. Elle tient. Tes mains sont collantes, Nina ? Un peu.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Nina a encore un peu de jus au doigt. C'est de la joie. Oui. Tu es contente. Et tu as partagé ta cerise. Tu as fini ton petit bout ? Oui. Nina essuie ses doigts sur l'herbe. Le cerisier fait encore de l'ombre.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nina tient la cerise contre sa paume, tout près. Je suis &lt;emphasis level="moderate"&gt;contente&lt;/emphasis&gt;. Tu le dis, Nina ? Oui, papa. Ses joues restent chaudes. Le ventre de Nina se desserre. On partage ? Tu veux tendre la cerise ? Oui, maman. Nina avance la cerise trop vite. Elle ouvre la bouche, trop large. Puis elle s'arrête. Nina refuse de foncer. Personne ne parle. Elle observe la cerise, un instant. Elle écoute le jardin. Nina tend la cerise vers papa. Papa prend un tout petit bout. Merci, Nina. Papa a vu le geste, sous l'arbre. Le jus est rouge. Il colle aux doigts, Nina ? Un peu, maman. Nina croque un tout petit bout. C'est sucré. Tu le sens, le sucre ? Oui, papa. Tes lèvres sont rouges, Nina ? Un peu, maman. Le ventre de Nina reste léger. Maman, un bout pour toi. Tu m'invites, Nina ? Oui. Maman attend, la main ouverte. La cerise est petite, Nina ? Oui, papa. Ils restent sous le cerisier. Elle tient. Tes mains sont collantes, Nina ? Un peu.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Emma a nommé sa joie. Elle a partagé avec papa. Être &lt;emphasis&gt;content&lt;/emphasis&gt;, c'est bien. [pause]</t>
+          <t>Nina tient la cerise contre sa paume, tout près. Je suis &lt;emphasis&gt;contente&lt;/emphasis&gt;. Tu le dis, Nina ? Oui, papa. Ses joues restent chaudes. Le ventre de Nina se desserre. On partage ? Tu veux tendre la cerise ? Oui, maman. Nina avance la cerise trop vite. Elle ouvre la bouche, trop large. Puis elle s'arrête. Nina refuse de foncer. Personne ne parle. Elle observe la cerise, un instant. Elle écoute le jardin. Nina tend la cerise vers papa. Papa prend un tout petit bout. Merci, Nina. Papa a vu le geste, sous l'arbre. Le jus est rouge. Il colle aux doigts, Nina ? Un peu, maman. Nina croque un tout petit bout. C'est sucré. Tu le sens, le sucre ? Oui, papa. Tes lèvres sont rouges, Nina ? Un peu, maman. Le ventre de Nina reste léger. Maman, un bout pour toi. Tu m'invites, Nina ? Oui. Maman attend, la main ouverte. La cerise est petite, Nina ? Oui, papa. Ils restent sous le cerisier. Elle tient. Tes mains sont collantes, Nina ? Un peu. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1639,7 +1672,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1647,10 +1680,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.18</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1673,30 +1706,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>content</t>
+          <t>contente</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1705,10 +1738,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1721,19 +1754,56 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=joie puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=elle_dit_je_suis_contente_elle_partage; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Nina a encore un peu de jus au doigt.
-enfant-f|C'est de la joie.
-maman|Oui. Tu es contente.
-maman|Et tu as partagé ta cerise.
-papa|Tu as fini ton petit bout ?
+          <t>narrateur|Nina tient la cerise contre sa paume, tout près.
+enfant-f|Je suis contente.
+papa|Tu le dis, Nina ?
+enfant-f|Oui, papa.
+narrateur|Ses joues restent chaudes.
+narrateur|Le ventre de Nina se desserre.
+enfant-f|On partage ?
+maman|Tu veux tendre la cerise ?
+enfant-f|Oui, maman.
+narrateur|Nina avance la cerise trop vite.
+narrateur|Elle ouvre la bouche, trop large.
+narrateur|Puis elle s'arrête.
+narrateur|Nina refuse de foncer.
+narrateur|Personne ne parle.
+narrateur|Elle observe la cerise, un instant.
+narrateur|Elle écoute le jardin.
+narrateur|Nina tend la cerise vers papa.
+narrateur|Papa prend un tout petit bout.
+papa|Merci, Nina.
+narrateur|Papa a vu le geste, sous l'arbre.
+enfant-f|Le jus est rouge.
+maman|Il colle aux doigts, Nina ?
+enfant-f|Un peu, maman.
+narrateur|Nina croque un tout petit bout.
+enfant-f|C'est sucré.
+papa|Tu le sens, le sucre ?
+enfant-f|Oui, papa.
+maman|Tes lèvres sont rouges, Nina ?
+enfant-f|Un peu, maman.
+narrateur|Le ventre de Nina reste léger.
+enfant-f|Maman, un bout pour toi.
+maman|Tu m'invites, Nina ?
 enfant-f|Oui.
-narrateur|Nina essuie ses doigts sur l'herbe.
-narrateur|Le cerisier fait encore de l'ombre.</t>
+narrateur|Maman attend, la main ouverte.
+papa|La cerise est petite, Nina ?
+enfant-f|Oui, papa.
+narrateur|Ils restent sous le cerisier.
+enfant-f|Elle tient.
+maman|Tes mains sont collantes, Nina ?
+enfant-f|Un peu.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>jardin</t>
         </is>
       </c>
     </row>
@@ -1760,17 +1830,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Nina pose le noyau dans le panier. Le jardin est calme. Une abeille s'éloigne. On rentre avec le panier ? Encore un peu, maman. On reste près de l'arbre. Tu as bien invité. Je suis contente. La joie est là, sous le cerisier. Nina pose sa main dans celle de papa. Ils restent encore un moment, sans se presser.</t>
+          <t>Le jus coule le long du doigt. Ça glisse ! Nina serre trop vite. Une goutte tombe dans l'herbe. Une autre, pour maman ! Une branche trop haute cache d'autres cerises, plus rouges. Un oiseau se pose sur la branche. Il va la prendre ! Nina avance les mains, trop vite. Puis elle s'arrête net. Nina refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe la cerise, un instant. Elle écoute le jardin, près du tuteur et du bois. Sur le bois, un éclat de tuteur luit. Là, sur le bois. Tu vois le point, Nina ? Oui, papa. Nina tient la cerise, sans se presser. Le jus arrête de couler. Pour toi, maman. Maman prend un tout petit bout. Il est sucré, Nina ? Oui, maman. L'oiseau reste sur la branche ? Oui, papa. L'oiseau picore plus haut, puis s'en va vers le portail. Il est parti. La cerise est restée, Nina ? Oui, avec nous. Nina essuie un peu de jus. Tes doigts sont rouges, Nina ? Un peu, papa. Le noyau apparaît, tout petit. Le noyau. Tu le poses, Nina ? Dans le panier. Nina pose le noyau dans le panier. Il est arrivé, le noyau ? Oui, papa. Le panier sent le sucre ? Un peu, maman.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Nina pose le noyau dans le panier. Le jardin est calme. Une abeille s'éloigne. On rentre avec le panier ? Encore un peu, maman. On reste près de l'arbre. Tu as bien invité. Je suis contente. La joie est là, sous le cerisier. Nina pose sa main dans celle de papa. Ils restent encore un moment, sans se presser.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le jus coule le long du doigt. Ça glisse ! Nina serre trop vite. Une goutte tombe dans l'herbe. Une autre, pour maman ! Une branche trop haute cache d'autres cerises, plus rouges. Un oiseau se pose sur la branche. Il va la prendre ! Nina avance les mains, trop vite. Puis elle s'arrête net. Nina refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe la cerise, un instant. Elle écoute le jardin, près du tuteur et du bois. Sur le bois, un &lt;emphasis level="moderate"&gt;éclat de tuteur&lt;/emphasis&gt; luit. Là, sur le bois. Tu vois le point, Nina ? Oui, papa. Nina tient la cerise, sans se presser. Le jus arrête de couler. Pour toi, maman. Maman prend un tout petit bout. Il est sucré, Nina ? Oui, maman. L'oiseau reste sur la branche ? Oui, papa. L'oiseau picore plus haut, puis s'en va vers le portail. Il est parti. La cerise est restée, Nina ? Oui, avec nous. Nina essuie un peu de jus. Tes doigts sont rouges, Nina ? Un peu, papa. Le noyau apparaît, tout petit. Le noyau. Tu le poses, Nina ? Dans le panier. Nina pose le noyau dans le panier. Il est arrivé, le noyau ? Oui, papa. Le panier sent le sucre ? Un peu, maman.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Emma essuie ses &lt;emphasis&gt;main&lt;/emphasis&gt;s. Le jardin est calme. Papa reste près d'elle. [pause]</t>
+          <t>Le jus coule le long du doigt. Ça glisse ! Nina serre trop vite. Une goutte tombe dans l'herbe. Une autre, pour maman ! Une branche trop haute cache d'autres cerises, plus rouges. Un oiseau se pose sur la branche. Il va la prendre ! Nina avance les mains, trop vite. Puis elle s'arrête net. Nina refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe la cerise, un instant. Elle écoute le jardin, près du tuteur et du bois. Sur le bois, un &lt;emphasis&gt;éclat de tuteur&lt;/emphasis&gt; luit. Là, sur le bois. Tu vois le point, Nina ? Oui, papa. Nina tient la cerise, sans se presser. Le jus arrête de couler. Pour toi, maman. Maman prend un tout petit bout. Il est sucré, Nina ? Oui, maman. L'oiseau reste sur la branche ? Oui, papa. L'oiseau picore plus haut, puis s'en va vers le portail. Il est parti. La cerise est restée, Nina ? Oui, avec nous. Nina essuie un peu de jus. Tes doigts sont rouges, Nina ? Un peu, papa. Le noyau apparaît, tout petit. Le noyau. Tu le poses, Nina ? Dans le panier. Nina pose le noyau dans le panier. Il est arrivé, le noyau ? Oui, papa. Le panier sent le sucre ? Un peu, maman. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1817,7 +1887,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1825,10 +1895,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.18</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1851,30 +1921,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>main</t>
+          <t>éclat de tuteur</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1883,10 +1953,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1897,19 +1967,61 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=jus_branche_oiseau_elle_refuse_de_foncer; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Nina pose le noyau dans le panier.
-narrateur|Le jardin est calme. Une abeille s'éloigne.
-maman|On rentre avec le panier ?
-enfant-f|Encore un peu, maman.
-papa|On reste près de l'arbre.
-papa|Tu as bien invité.
-enfant-f|Je suis contente.
-maman|La joie est là, sous le cerisier.
-narrateur|Nina pose sa main dans celle de papa.
-narrateur|Ils restent encore un moment, sans se presser.</t>
+          <t>narrateur|Le jus coule le long du doigt.
+enfant-f|Ça glisse !
+narrateur|Nina serre trop vite.
+narrateur|Une goutte tombe dans l'herbe.
+enfant-f|Une autre, pour maman !
+narrateur|Une branche trop haute cache d'autres cerises, plus rouges.
+narrateur|Un oiseau se pose sur la branche.
+enfant-f|Il va la prendre !
+narrateur|Nina avance les mains, trop vite.
+narrateur|Puis elle s'arrête net.
+narrateur|Nina refuse de foncer, cette fois.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Personne ne dit la suite.
+narrateur|Elle observe la cerise, un instant.
+narrateur|Elle écoute le jardin, près du tuteur et du bois.
+narrateur|Sur le bois, un éclat de tuteur luit.
+enfant-f|Là, sur le bois.
+papa|Tu vois le point, Nina ?
+enfant-f|Oui, papa.
+narrateur|Nina tient la cerise, sans se presser.
+narrateur|Le jus arrête de couler.
+enfant-f|Pour toi, maman.
+narrateur|Maman prend un tout petit bout.
+maman|Il est sucré, Nina ?
+enfant-f|Oui, maman.
+papa|L'oiseau reste sur la branche ?
+enfant-f|Oui, papa.
+narrateur|L'oiseau picore plus haut, puis s'en va vers le portail.
+enfant-f|Il est parti.
+maman|La cerise est restée, Nina ?
+enfant-f|Oui, avec nous.
+narrateur|Nina essuie un peu de jus.
+papa|Tes doigts sont rouges, Nina ?
+enfant-f|Un peu, papa.
+narrateur|Le noyau apparaît, tout petit.
+enfant-f|Le noyau.
+maman|Tu le poses, Nina ?
+enfant-f|Dans le panier.
+narrateur|Nina pose le noyau dans le panier.
+papa|Il est arrivé, le noyau ?
+enfant-f|Oui, papa.
+maman|Le panier sent le sucre ?
+enfant-f|Un peu, maman.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>jardin,cerisier</t>
         </is>
       </c>
     </row>
@@ -1936,17 +2048,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>J'ai dit : je suis contente. On a partagé la cerise. Bravo, Nina.</t>
+          <t>Ils restent près du cerisier. On a partagé, papa. Tu l'as vu, toi ? Oui, près de l'arbre. On est bien, ici. Nina tapote le bois du tuteur. Il a une trace de jus. Tu la vois, la trace ? Oui, maman. Le portail attend, Nina. Oui, un peu ouvert. Ça sent le sucre, un peu tiède. Et le bois, maman. Oui, dans l'air. Le jardin est calme, Nina ? Oui, papa. Le panier reste près de l'herbe. Un éclat de tuteur tient sur le bois.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>J'ai dit : je suis contente. On a partagé la cerise. Bravo, Nina.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près du cerisier. On a partagé, papa. Tu l'as vu, toi ? Oui, près de l'arbre. On est bien, ici. Nina tapote le bois du tuteur. Il a une trace de jus. Tu la vois, la trace ? Oui, maman. Le portail attend, Nina. Oui, un peu ouvert. Ça sent le sucre, un peu tiède. Et le bois, maman. Oui, dans l'air. Le jardin est calme, Nina ? Oui, papa. Le panier reste près de l'herbe. Un &lt;emphasis level="moderate"&gt;éclat de tuteur&lt;/emphasis&gt; tient sur le bois.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près du cerisier. On a partagé, papa. Tu l'as vu, toi ? Oui, près de l'arbre. On est bien, ici. Nina tapote le bois du tuteur. Il a une trace de jus. Tu la vois, la trace ? Oui, maman. Le portail attend, Nina. Oui, un peu ouvert. Ça sent le sucre, un peu tiède. Et le bois, maman. Oui, dans l'air. Le jardin est calme, Nina ? Oui, papa. Le panier reste près de l'herbe. Un &lt;emphasis&gt;éclat de tuteur&lt;/emphasis&gt; tient sur le bois.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -1993,7 +2105,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2001,10 +2113,10 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.26</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2013,12 +2125,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2027,17 +2139,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de tuteur</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2046,11 +2162,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2059,26 +2175,45 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_bois; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-f|J'ai dit : je suis contente.
-enfant-f|On a partagé la cerise.
-papa|Bravo, Nina.</t>
+          <t>narrateur|Ils restent près du cerisier.
+enfant-f|On a partagé, papa.
+papa|Tu l'as vu, toi ?
+enfant-f|Oui, près de l'arbre.
+maman|On est bien, ici.
+narrateur|Nina tapote le bois du tuteur.
+enfant-f|Il a une trace de jus.
+maman|Tu la vois, la trace ?
+enfant-f|Oui, maman.
+papa|Le portail attend, Nina.
+enfant-f|Oui, un peu ouvert.
+narrateur|Ça sent le sucre, un peu tiède.
+enfant-f|Et le bois, maman.
+maman|Oui, dans l'air.
+papa|Le jardin est calme, Nina ?
+enfant-f|Oui, papa.
+narrateur|Le panier reste près de l'herbe.
+narrateur|Un éclat de tuteur tient sur le bois.</t>
         </is>
       </c>
     </row>
@@ -2099,7 +2234,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2163,6 +2298,13 @@
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>